<commit_message>
web scraping mercado livre
</commit_message>
<xml_diff>
--- a/produtos.xlsx
+++ b/produtos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,6 +455,1410 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Urna Acrílico Transparente Piramide 20x20x12cm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolivre.com.br/mclics/clicks/external/MLB/count?a=O%2FFxIS0WT0XORBaUw3Vaj4ZgrO21qO0nG6JH1RvAD9%2BE4E1B1ffZDXbLFLLE6LVBTDbGCghG5yRfDg9B4KhQQLhVHasJbcPjmjesFQ6U91m%2BjhpmnUBGtnEXF%2FTQ4BuJMqztd5knneimT46BqF%2BqBPo7KvLcRjGpiQf7tyt%2Ba8co7%2Bg3wd%2BTpLjx2XzdGT9DAXN8yrayzDPqh1ETb3Q0aEyECG%2FgQ3qQlnOMDKV7i5bPu4e11wijhF6kZp49AyrUY9rX%2FrhdojgQeCuiohCyijhqcOUX1Yi7evEFOgWDanO9D9x6xjkqHzx9h1%2B4qGb4Yie68vhZ8M0Gr4%2FoD8nWDOkv3XXTZdd2AvUJiKGq%2FV3TjxcfCooKEutUnzWLkAFUm806ktDsSFk0ScvFqxAAxBTuDzgEjolp5c3lfX39dXI0eWzM7iDuIKi7A%2BQEGsuTsMcUDggaJR8KMw1wjUUuhWYYg1213JYSO%2Fv1AjXpRcoWgHaqcTzkT0cVeC3%2FdyM16kthoM15%2BiCKW8OpRoz6cSmbKA5RQLS%2F3N%2FOg2UBTW1e68UixSq39%2BMP7whZ9KDqnxpV%2Fl3u4ml61tbYill6BYwO2EIo%2FJKxAxFQ6iCNxL3CkMTiOc%2Fg1GWocM8ZaIHz%2FTreOcupoeQvjsOWHiAv8Bc8c%2BF%2BRrRgKTDGUFoEEJ46SmT5wY9z%2FdqWQKoD6tQBp1MyLjtbX8K%2FdXeTv2KriIWY8dGn5UugkUVq3fJFzlAQ7T6x4NvxN63dUmLg1hr3KpRVIA%3D%3D&amp;rb=x#polycard_client=search-nordic&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10 Caixas Para 100 Doces Com Berço 35x35x5 Cm - Branco</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://click1.mercadolivre.com.br/mclics/clicks/external/MLB/count?a=NHnZq%2BEv3Ob9Kl2hkjHA2wLNGxVYSEMtAMUI6DG%2F2brsk34Ztho2qNseKJeX8KX4NM4SuA73AgVS8%2BY2ArrEzAj5gYAmN7hIF2iUB4HcQ%2BfHXPyushaa0yqidr7reDmHRdI2JrKpE9U63%2Bq2FRrUQg%2FEI5PYlI7bc3HW8Ut1XBupJ4zeEiNNq3QUGC76ItOc8ozwWL2Ke5NZwWh2leOspmClqbiqVrJPLBusPXkLI79IikpR6qxwfOLgpEiuAbNZxyCPvRqs%2Bvh0CvY13SvXVQvaSUIwpn9CBopGn2HH9B2fnvwldS9NUXS2mV9MkbTzjeZCX%2BhvuP93N8pj0vn%2FME1Zka3TlR1mkvVq896E3wLGcV%2FS%2F6L1cQFMBX25TIt87L6BaeTmOR0RekHlfeXKPvbOUDBrmBpzjaWb2CKGqJH9%2BFS%2BtWd8j9HUHdtUb7eJv26Bxkq1%2Bbl6IKk0ZbgrWRdddKRlZ13fucHWMCnZ1NVn5jZOVDY7aBaXw1o%2Bg%2F7ih4U1wLtu0XLabDfD9gaJlrPLjszNc%2Fd0vgch3bD92vLYpCirhEkLwEWn0ThyEeLy5a8XYZWCvSDlt32EaXxEFFmUd6N9wvJKZvrCKy6C5WYHnN4Ph6KMcLr%2FUcyXCJTRwo6GK92gipcEdMr5hcZpYQcIL5vYca48MzXbFDso%2FN22k98cqxv6%2B9cBF5mZFaJrIegVj6uuRc2bUMP%2BRTNnPi9BQvjDedyCplqMwP0GZ4MhKZR7DeRz0iInGDfdUHPMIbf02%2BGYtOQr&amp;rb=x#polycard_client=search-nordic&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>POP Imports kit 10 fita adesiva transparente 500m x 4.5cm</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/pop-imports-kit-10-fita-adesiva-transparente-500m-x-45cm/p/MLB25300768#polycard_client=search-nordic&amp;searchVariation=MLB25300768&amp;wid=MLB3657966981&amp;position=5&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Urna Pirâmide De Acrílico - 30 Cm - Pronta</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/urna-pirmide-de-acrilico-30-cm-pronta/p/MLB45360312#polycard_client=search-nordic&amp;searchVariation=MLB45360312&amp;wid=MLB3958682731&amp;position=6&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Kit 10 Caixas Papelão Mudança Embalagem 60x40x40 Grande</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-10-caixas-papelo-mudanca-embalagem-60x40x40-grande/p/MLB36222806#polycard_client=search-nordic&amp;searchVariation=MLB36222806&amp;wid=MLB4795077986&amp;position=4&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sabão em pó lavagem perfeita ativo concentrado 2,2kg Omo</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/sabo-em-po-lavagem-perfeita-ativo-concentrado-22kg-omo/p/MLB17001105#polycard_client=search-nordic&amp;searchVariation=MLB17001105&amp;wid=MLB2910494284&amp;position=9&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Detergente Unik Toys Secante e Abrilhantador Brisa de Limão em pó limão em caixa 1 kg</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/detergente-unik-toys-secante-e-abrilhantador-brisa-de-limo-em-po-limo-em-caixa-1-kg/p/MLB16949080#polycard_client=search-nordic&amp;searchVariation=MLB16949080&amp;wid=MLB3834200311&amp;position=3&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Piscina Inflável Fun Redonda 1400L com Kit Reparo Mor</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/piscina-inflavel-fun-redonda-1400l-com-kit-reparo-mor/p/MLB10923645#polycard_client=search-nordic&amp;searchVariation=MLB10923645&amp;wid=MLB2062536329&amp;position=15&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>279</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Kit 3 Caixas Organizadoras Transparente 6 Litros Uninjet</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-3-caixas-organizadoras-transparente-6-litros-uninjet/p/MLB27250231#polycard_client=search-nordic&amp;searchVariation=MLB27250231&amp;wid=MLB4555645346&amp;position=10&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>100 Caixinhas Para Canecas Sublimaticas 325 Ml (branca)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/100-caixinhas-para-canecas-sublimaticas-325-ml-branca/p/MLB28562480#polycard_client=search-nordic&amp;searchVariation=MLB28562480&amp;wid=MLB4918867032&amp;position=14&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Caixa Caixinha De Som Bluetooth Portatil Radio Fm Potente Cor Preto Grasep DD-3138</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-caixinha-de-som-bluetooth-portatil-radio-fm-potente-cor-preto-grasep-dd-3138/p/MLB26085607#polycard_client=search-nordic&amp;searchVariation=MLB26085607&amp;wid=MLB4161118144&amp;position=18&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Caixa Organizadora Multiuso Helsim Cesto Tampa Com 45 Litros Grande Cor Preto</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-organizadora-multiuso-helsim-cesto-tampa-com-45-litros-grande-cor-preto/p/MLB29076161#polycard_client=search-nordic&amp;searchVariation=MLB29076161&amp;wid=MLB5163916924&amp;position=13&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Caixa de Som Bluetooth PartyBox Stage 320 JBL BLPBSTAGE320BR Preta 110V/220V</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-de-som-bluetooth-partybox-stage-320-jbl-blpbstage320br-preta-110v220v/p/MLB36336899#polycard_client=search-nordic&amp;searchVariation=MLB36336899&amp;wid=MLB3849952029&amp;position=8&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>3.800</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tiras Para Medição de Glicose Accu chek Active Caixa com 50 Un</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/tiras-para-medico-de-glicose-accu-chek-active-caixa-com-50-un/p/MLB25754310#polycard_client=search-nordic&amp;searchVariation=MLB25754310&amp;wid=MLB3625890261&amp;position=16&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>50 Caixas De Papelão 16x11x6 Cm Batom, Maquiagem, iPhone</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/50-caixas-de-papelo-16x11x6-cm-batom-maquiagem-iphone/p/MLB29351427#polycard_client=search-nordic&amp;searchVariation=MLB29351427&amp;wid=MLB3691549799&amp;position=11&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Kit 3 Livros Fake Decoraçao Caixas Porta Objeto Decorativo Cor Design Rústico</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-3-livros-fake-decoracao-caixas-porta-objeto-decorativo-cor-design-rustico/p/MLB34961946#polycard_client=search-nordic&amp;searchVariation=MLB34961946&amp;wid=MLB3913712283&amp;position=7&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Kit 10 fita adesiva embalagem durex caixa 45mm x 500m transparente Solução &amp; Cia</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-10-fita-adesiva-embalagem-durex-caixa-45mm-x-500m-transparente-soluco-cia/p/MLB25144306#polycard_client=search-nordic&amp;searchVariation=MLB25144306&amp;wid=MLB3748497737&amp;position=17&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cartas de Pokémon Box Display Coroa Estelar Hydrapple Copag em Portugués</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/cartas-de-pokemon-box-display-coroa-estelar-hydrapple-copag-em-portugues/p/MLB41347145#polycard_client=search-nordic&amp;searchVariation=MLB41347145&amp;wid=MLB3937362097&amp;position=21&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10 Caixa Caixinha 15x15x5 Mdf Crú Padrinhos Lembrancinha Tt</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/10-caixa-caixinha-15x15x5-mdf-cru-padrinhos-lembrancinha-tt/p/MLB28757269#polycard_client=search-nordic&amp;searchVariation=MLB28757269&amp;wid=MLB3810258853&amp;position=20&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Kit 10 rolo fita adesiva 45x500 metros transparente Zi Store</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-10-rolo-fita-adesiva-45x500-metros-transparente-zi-store/p/MLB25257716#polycard_client=search-nordic&amp;searchVariation=MLB25257716&amp;wid=MLB4131655968&amp;position=12&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Echo Dot 5ª Geração Alto-falante De 1,73 Preto Amazon B09B8VGCR8 Bivolt</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/echo-dot-5-geraco-alto-falante-de-173-preto-amazon-b09b8vgcr8-bivolt/p/MLB27190731#polycard_client=search-nordic&amp;searchVariation=MLB27190731&amp;wid=MLB4355876114&amp;position=22&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>342</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tramontina 43800005 caixa para ferramentas sanfonada com 5 gavetas</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/tramontina-43800005-caixa-para-ferramentas-sanfonada-com-5-gavetas/p/MLB22367713#polycard_client=search-nordic&amp;searchVariation=MLB22367713&amp;wid=MLB3897718148&amp;position=25&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Beethoven Agropet caixa de abelha langstroth com 2 melgueiras em eucalipto rosa</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/beethoven-agropet-caixa-de-abelha-langstroth-com-2-melgueiras-em-eucalipto-rosa/p/MLB30396012#polycard_client=search-nordic&amp;searchVariation=MLB30396012&amp;wid=MLB5061299850&amp;position=19&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Caixa Organizadora Rattan 70 Litros Preto</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-organizadora-rattan-70-litros-preto/p/MLB27093149#polycard_client=search-nordic&amp;searchVariation=MLB27093149&amp;wid=MLB4688547284&amp;position=23&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Microcânula 22g X 50mm Caixa Com 10 Unidades - Smart Gr</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/microcnula-22g-x-50mm-caixa-com-10-unidades-smart-gr/p/MLB36188176#polycard_client=search-nordic&amp;searchVariation=MLB36188176&amp;wid=MLB5192632724&amp;position=24&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>20 Rolos Fita Adesiva Durex Embalagem Rolo Transparente 500m</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/20-rolos-fita-adesiva-durex-embalagem-rolo-transparente-500m/p/MLB32822781#polycard_client=search-nordic&amp;searchVariation=MLB32822781&amp;wid=MLB4651463680&amp;position=36&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Urna Piramide Idealle Acrilicos Piramide 40 Cm</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/urna-piramide-idealle-acrilicos-piramide-40-cm/p/MLB44556241#polycard_client=search-nordic&amp;searchVariation=MLB44556241&amp;wid=MLB3953959439&amp;position=38&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Kit 4 Caixas Organizadoras Com Tampa E Trava 56 Litros Grande Resistente Preta</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-4-caixas-organizadoras-com-tampa-e-trava-56-litros-grande-resistente-preta/p/MLB44122314#polycard_client=search-nordic&amp;searchVariation=MLB44122314&amp;wid=MLB3956029015&amp;position=26&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Caixa De Som Bluetooth 40w Ipx6 Prova D'água Cor Preto 110V/220V Fam A042</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-de-som-bluetooth-40w-ipx6-prova-dagua-cor-preto-110v220v-fam-a042/p/MLB23442240#polycard_client=search-nordic&amp;searchVariation=MLB23442240&amp;wid=MLB5244759256&amp;position=28&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Kit 10 Caixa Papelão 50x30x40 Grande Mudança S Sedex</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-10-caixa-papelo-50x30x40-grande-mudanca-s-sedex/p/MLB29315167#polycard_client=search-nordic&amp;searchVariation=MLB29315167&amp;wid=MLB5179548302&amp;position=27&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>25 Caixas De Papelão P/ Correios Pac Sedex 30x20x20 Cm</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-1961820976-25-caixas-de-papelo-p-correios-pac-sedex-30x20x20-cm-_JM#polycard_client=search-nordic&amp;position=50&amp;search_layout=stack&amp;type=item&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Caixa Gordura Tigre  Com tampa</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-gordura-tigre-com-tampa/p/MLB36041636#polycard_client=search-nordic&amp;searchVariation=MLB36041636&amp;wid=MLB3882056777&amp;position=29&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>316</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Organizador multiuso caixa preta 56 litros com tampa trava cor preto</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/organizador-multiuso-caixa-preta-56-litros-com-tampa-trava-cor-preto/p/MLB29366528#polycard_client=search-nordic&amp;searchVariation=MLB29366528&amp;wid=MLB3822146963&amp;position=30&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Caixa Porta Lâminas Para 100 Lâminas</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-porta-lminas-para-100-lminas/p/MLB24689805#polycard_client=search-nordic&amp;searchVariation=MLB24689805&amp;wid=MLB3686664245&amp;position=31&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Agulha Lebel 32g 4mm - Caixa Com 100 Unidades</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/agulha-lebel-32g-4mm-caixa-com-100-unidades/p/MLB32399381#polycard_client=search-nordic&amp;searchVariation=MLB32399381&amp;wid=MLB3640753335&amp;position=33&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Caixa De Som Bluetooth Flip 6 30w Rms Jbl Cor Preto 110V/220V</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-de-som-bluetooth-flip-6-30w-rms-jbl-cor-preto-110v220v/p/MLB18930466#polycard_client=search-nordic&amp;searchVariation=MLB18930466&amp;wid=MLB3452479497&amp;position=32&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>865</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Caixas Papelão Modelo Correios Sedex 25x25x25 100 Unid</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixas-papelo-modelo-correios-sedex-25x25x25-100-unid/p/MLB44301192#polycard_client=search-nordic&amp;searchVariation=MLB44301192&amp;wid=MLB3922247655&amp;position=34&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>439</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Caixa Organizadora Multiuso Plástica 56 Litros Kit 2 Peças Cor Preto</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-organizadora-multiuso-plastica-56-litros-kit-2-pecas-cor-preto/p/MLB29388813#polycard_client=search-nordic&amp;searchVariation=MLB29388813&amp;wid=MLB5105164618&amp;position=35&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Gedore Robust Jogo De Ferramentas Oficina Master Maleta 178 Itens cor preto e laranja</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/gedore-robust-jogo-de-ferramentas-oficina-master-maleta-178-itens-cor-preto-e-laranja/p/MLB21017963#polycard_client=search-nordic&amp;searchVariation=MLB21017963&amp;wid=MLB3872241023&amp;position=37&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1.081</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Play Embalagens kit 5 caixas papelão 60x40x40cm kraft</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/play-embalagens-kit-5-caixas-papelo-60x40x40cm-kraft/p/MLB34729931#polycard_client=search-nordic&amp;searchVariation=MLB34729931&amp;wid=MLB5097578772&amp;position=39&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Agulha Lebel 32g 4mm - Caixa Com 100 Unidades</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/agulha-lebel-32g-4mm-caixa-com-100-unidades/p/MLB33068649#polycard_client=search-nordic&amp;searchVariation=MLB33068649&amp;wid=MLB4454921846&amp;position=40&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Kit 2 Caixa Organizadora Plástica C/ Tampa Rattan 40l Preto Liso</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-2-caixa-organizadora-plastica-c-tampa-rattan-40l-preto-liso/p/MLB27093894#polycard_client=search-nordic&amp;searchVariation=MLB27093894&amp;wid=MLB3880920917&amp;position=41&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Urna Acrílico Transparente Piramide 20x20x12cm</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-4746023154-urna-acrilico-transparente-piramide-20x20x12cm-_JM#polycard_client=search-nordic&amp;position=51&amp;search_layout=stack&amp;type=item&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Seringa Descartável 10ml Bico Lock Caixa Com 100 Unidades Descarpack</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/seringa-descartavel-10ml-bico-lock-caixa-com-100-unidades-descarpack/p/MLB23416639#polycard_client=search-nordic&amp;searchVariation=MLB23416639&amp;wid=MLB3360637849&amp;position=42&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Echo Pop Smart Speaker Amazon Cor Preto C2H4R9</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/echo-pop-smart-speaker-amazon-cor-preto-c2h4r9/p/MLB23995388#polycard_client=search-nordic&amp;searchVariation=MLB23995388&amp;wid=MLB5237682352&amp;position=43&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>254</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Caixa 60 Rolos Fita Adesiva Transparente 45mm X 100 Mts</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/caixa-60-rolos-fita-adesiva-transparente-45mm-x-100-mts/p/MLB32725481#polycard_client=search-nordic&amp;searchVariation=MLB32725481&amp;wid=MLB3823552911&amp;position=44&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Fio Fada Cordão De Led 2m 20 Leds 3 Funções Bateria Branco Quente Cor das luzes Amarelo Bateria Cabo Branco Wincy Fio de Fada</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/fio-fada-cordo-de-led-2m-20-leds-3-funcoes-bateria-branco-quente-cor-das-luzes-amarelo-bateria-cabo-branco-wincy-fio-de-fada/p/MLB28896064#polycard_client=search-nordic&amp;searchVariation=MLB28896064&amp;wid=MLB4700221578&amp;position=48&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>10 Caixas Para 100 Doces Com Berço 35x35x5 Cm - Branco</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://produto.mercadolivre.com.br/MLB-2744787639-10-caixas-para-100-doces-com-berco-35x35x5-cm-branco-_JM#polycard_client=search-nordic&amp;position=52&amp;search_layout=stack&amp;type=item&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Kit 3 Caixas Organizadoras Transparente 3 Litros Pp Uninjet Liso</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/kit-3-caixas-organizadoras-transparente-3-litros-pp-uninjet-liso/p/MLB32598844#polycard_client=search-nordic&amp;searchVariation=MLB32598844&amp;wid=MLB3746714741&amp;position=45&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Leite UHT integral 1 Litro Italac</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/leite-uht-integral-1-litro-italac/p/MLB18311507#polycard_client=search-nordic&amp;searchVariation=MLB18311507&amp;wid=MLB3700835041&amp;position=49&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Envelope Plastico Correios De Seguranca Cinza 12x18 1000 Uni</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/envelope-plastico-correios-de-seguranca-cinza-12x18-1000-uni/p/MLB36299907#polycard_client=search-nordic&amp;searchVariation=MLB36299907&amp;wid=MLB3676655585&amp;position=46&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Maleta Organização Decorativa Grande 39cm Com Fecho E Alça</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://www.mercadolivre.com.br/maleta-organizaco-decorativa-grande-39cm-com-fecho-e-alca/p/MLB30902071#polycard_client=search-nordic&amp;searchVariation=MLB30902071&amp;wid=MLB3583235189&amp;position=47&amp;search_layout=stack&amp;type=product&amp;tracking_id=058b448e-2554-4ab3-bfb6-488bd0471c94&amp;sid=search</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>R$</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>